<commit_message>
🤖 AI Trader update — 22 Mar 2026
- Week Trade: NET / MRVL (งบ $200)
- NET $120: Entry $213.50 | TP $220/$226/$232 | SL $208 | R/R 1:2.4
- MRVL $80: Entry $87.50 | TP $91.50/$94.50/$97.50 | SL $84.50 | R/R 1:2.0
- Redesign AI Trading tab: sub-tab per stock + visual cards
- Excel Sheet 2: col S filter for active trades

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/รายรับ_รายจ่าย_ประจำปี.xlsx
+++ b/รายรับ_รายจ่าย_ประจำปี.xlsx
@@ -1451,7 +1451,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="710">
+  <cellXfs count="712">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -3567,6 +3567,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="65" fillId="36" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -5781,7 +5787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O69"/>
+  <dimension ref="A1:O59"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="35" customWidth="1" style="349" min="1" max="1"/>
@@ -7662,16 +7668,6 @@
       <c r="J59" s="427" t="n"/>
       <c r="K59" s="427" t="n"/>
     </row>
-    <row r="60"/>
-    <row r="61"/>
-    <row r="62"/>
-    <row r="63"/>
-    <row r="64"/>
-    <row r="65"/>
-    <row r="66"/>
-    <row r="67"/>
-    <row r="68"/>
-    <row r="69"/>
   </sheetData>
   <mergeCells count="45">
     <mergeCell ref="H53:I53"/>
@@ -7763,7 +7759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:W11"/>
+  <dimension ref="A1:S10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="349" min="1" max="1"/>
@@ -7789,7 +7785,7 @@
     <row r="1" ht="24" customHeight="1" s="350">
       <c r="A1" s="456" t="inlineStr">
         <is>
-          <t>🤖  AI Trading — แผนการลงทุน Week Trade (ถือ 3-5 วัน)  |  งบประมาณ: $140 (~5,000฿)  |  อัปเดต: 21 Mar 2026  |  ⚡ เปลี่ยนจาก CIEN → MRVL (chart setup ดีกว่า)</t>
+          <t>🤖 AI Trading — แผนการลงทุน Week Trade (ถือ 3-5 วัน)  |  งบประมาณ: $200  |  อัปเดต: 22 Mar 2026  |  ⚡ Week Trade: NET / MRVL</t>
         </is>
       </c>
       <c r="B1" s="438" t="n"/>
@@ -7815,7 +7811,7 @@
       </c>
       <c r="B2" s="438" t="n"/>
       <c r="C2" s="458" t="n">
-        <v>10000</v>
+        <v>200</v>
       </c>
       <c r="D2" s="457" t="inlineStr">
         <is>
@@ -7960,14 +7956,6 @@
           <t>สถานะ</t>
         </is>
       </c>
-      <c r="T3" s="464" t="n"/>
-      <c r="U3" s="464" t="n"/>
-      <c r="V3" s="464" t="n"/>
-      <c r="W3" s="463" t="inlineStr">
-        <is>
-          <t>📊 Analysis Summary</t>
-        </is>
-      </c>
     </row>
     <row r="4" ht="309.75" customHeight="1" s="350">
       <c r="A4" s="465" t="n">
@@ -7975,119 +7963,117 @@
       </c>
       <c r="B4" s="466" t="inlineStr">
         <is>
+          <t>NET</t>
+        </is>
+      </c>
+      <c r="C4" s="467" t="inlineStr">
+        <is>
+          <t>Cloudflare, Inc.</t>
+        </is>
+      </c>
+      <c r="D4" s="468" t="inlineStr">
+        <is>
+          <t>N/M</t>
+        </is>
+      </c>
+      <c r="E4" s="469" t="n">
+        <v>213.5</v>
+      </c>
+      <c r="F4" s="470" t="n">
+        <v>0.5581</v>
+      </c>
+      <c r="G4" s="469" t="n">
+        <v>120</v>
+      </c>
+      <c r="H4" s="471" t="n">
+        <v>208</v>
+      </c>
+      <c r="I4" s="472" t="n">
+        <v>-0.026</v>
+      </c>
+      <c r="J4" s="471" t="n">
+        <v>220</v>
+      </c>
+      <c r="K4" s="473" t="n">
+        <v>226</v>
+      </c>
+      <c r="L4" s="474" t="n">
+        <v>232</v>
+      </c>
+      <c r="M4" s="475" t="inlineStr">
+        <is>
+          <t>1:2.4</t>
+        </is>
+      </c>
+      <c r="N4" s="476" t="n"/>
+      <c r="O4" s="477" t="inlineStr">
+        <is>
+          <t>Single entry — EMA50 1H + RSI 1H oversold | TP1 40% → TP2 40% → TP3 20% | SL -2.6%</t>
+        </is>
+      </c>
+      <c r="P4" s="478" t="n"/>
+      <c r="Q4" s="479" t="n"/>
+      <c r="R4" s="480" t="n"/>
+      <c r="S4" s="481" t="n"/>
+    </row>
+    <row r="5" ht="75" customHeight="1" s="350">
+      <c r="A5" s="484" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="485" t="inlineStr">
+        <is>
           <t>MRVL</t>
         </is>
       </c>
-      <c r="C4" s="467" t="inlineStr">
+      <c r="C5" s="486" t="inlineStr">
         <is>
           <t>Marvell Technology, Inc.</t>
         </is>
       </c>
-      <c r="D4" s="468" t="n">
-        <v>35</v>
-      </c>
-      <c r="E4" s="469" t="n">
-        <v>62.87</v>
-      </c>
-      <c r="F4" s="470">
-        <f>G4/E4</f>
-        <v/>
-      </c>
-      <c r="G4" s="469" t="n">
-        <v>140</v>
-      </c>
-      <c r="H4" s="471">
-        <f>E4*(1+I4)</f>
-        <v/>
-      </c>
-      <c r="I4" s="472" t="n">
-        <v>-0.05</v>
-      </c>
-      <c r="J4" s="471">
-        <f>E4*(1+K4)</f>
-        <v/>
-      </c>
-      <c r="K4" s="473" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="L4" s="474">
-        <f>ABS(K4/I4)</f>
-        <v/>
-      </c>
-      <c r="M4" s="475">
-        <f>G4*K4</f>
-        <v/>
-      </c>
-      <c r="N4" s="476">
-        <f>G4*I4</f>
-        <v/>
-      </c>
-      <c r="O4" s="477" t="inlineStr">
-        <is>
-          <t>🔄 เปลี่ยนจาก CIEN (chart setup ดีกว่า)
-─────────────────────
-📌 แบ่ง 3 ไม้ (งบ ~$140 / 5,000฿)
-ไม้ 1: $56 → เข้าตอนนี้ EMA100(1H) $87.23
-ไม้ 2: $49 → Dip ที่ EMA200(1H) $85.09
-ไม้ 3: $35 → Breakout เหนือ EMA50 $88.64
-─────────────────────
-🎯 TP1 +5% $91.9 | TP2 +8% $94.5 | TP3 +12% $98
-🛑 Cut Loss -5% ($83) ต่ำกว่า EMA200(1H)
-📊 1D RSI=59 (neutral✅) | 1H RSI=39 (near oversold✅)
-⚡ เหตุผล: EMA100 support ชัด + RSI1H ใกล้ oversold + 1D โครงสร้างดี</t>
-        </is>
-      </c>
-      <c r="P4" s="478" t="n"/>
-      <c r="Q4" s="479">
-        <f>IF(AND(ISNUMBER(P4),P4&gt;0),P4-G4,"")</f>
-        <v/>
-      </c>
-      <c r="R4" s="480">
-        <f>IF(AND(ISNUMBER(P4),P4&gt;0),(P4-G4)/G4,"")</f>
-        <v/>
-      </c>
-      <c r="S4" s="481">
-        <f>IF(AND(ISNUMBER(P4),P4&gt;0),IF(P4-G4&gt;0,"✅ กำไร","🔴 ขาดทุน"),"")</f>
-        <v/>
-      </c>
-      <c r="T4" s="482" t="n"/>
-      <c r="U4" s="482" t="n"/>
-      <c r="V4" s="482" t="n"/>
-      <c r="W4" s="483" t="inlineStr"/>
-    </row>
-    <row r="5" ht="75" customHeight="1" s="350">
-      <c r="A5" s="484" t="n"/>
-      <c r="B5" s="485" t="n"/>
-      <c r="C5" s="486" t="n"/>
-      <c r="D5" s="487" t="n"/>
-      <c r="E5" s="488" t="n"/>
-      <c r="F5" s="489" t="n"/>
-      <c r="G5" s="490" t="n"/>
-      <c r="H5" s="491" t="n"/>
-      <c r="I5" s="492" t="n"/>
-      <c r="J5" s="493" t="n"/>
-      <c r="K5" s="494" t="n"/>
-      <c r="L5" s="495" t="n"/>
-      <c r="M5" s="496" t="n"/>
+      <c r="D5" s="487" t="inlineStr">
+        <is>
+          <t>N/M</t>
+        </is>
+      </c>
+      <c r="E5" s="488" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="F5" s="489" t="n">
+        <v>0.9091</v>
+      </c>
+      <c r="G5" s="490" t="n">
+        <v>80</v>
+      </c>
+      <c r="H5" s="491" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="I5" s="492" t="n">
+        <v>-0.034</v>
+      </c>
+      <c r="J5" s="493" t="n">
+        <v>91.5</v>
+      </c>
+      <c r="K5" s="494" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="L5" s="495" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="M5" s="496" t="inlineStr">
+        <is>
+          <t>1:2.0</t>
+        </is>
+      </c>
       <c r="N5" s="497" t="n"/>
-      <c r="O5" s="498" t="n"/>
+      <c r="O5" s="498" t="inlineStr">
+        <is>
+          <t>Confirm entry: dip $86.50-87.50 RSI&lt;40 OR breakout close&gt;EMA20($88.50) | TP1 50% → TP2 30% → TP3 20% | SL -3.4%</t>
+        </is>
+      </c>
       <c r="P5" s="478" t="n"/>
-      <c r="Q5" s="479">
-        <f>IF(AND(ISNUMBER(P5),P5&gt;0),P5-G5,"")</f>
-        <v/>
-      </c>
-      <c r="R5" s="480">
-        <f>IF(AND(ISNUMBER(P5),P5&gt;0),(P5-G5)/G5,"")</f>
-        <v/>
-      </c>
-      <c r="S5" s="481">
-        <f>IF(AND(ISNUMBER(P5),P5&gt;0),IF(P5-G5&gt;0,"✅ กำไร","🔴 ขาดทุน"),"")</f>
-        <v/>
-      </c>
-      <c r="T5" s="482" t="n"/>
-      <c r="U5" s="482" t="n"/>
-      <c r="V5" s="482" t="n"/>
-      <c r="W5" s="482" t="n"/>
+      <c r="Q5" s="479" t="n"/>
+      <c r="R5" s="480" t="n"/>
+      <c r="S5" s="481" t="n"/>
     </row>
     <row r="6" ht="75" customHeight="1" s="350">
       <c r="A6" s="484" t="n"/>
@@ -8106,22 +8092,9 @@
       <c r="N6" s="497" t="n"/>
       <c r="O6" s="498" t="n"/>
       <c r="P6" s="478" t="n"/>
-      <c r="Q6" s="479">
-        <f>IF(AND(ISNUMBER(P6),P6&gt;0),P6-G6,"")</f>
-        <v/>
-      </c>
-      <c r="R6" s="480">
-        <f>IF(AND(ISNUMBER(P6),P6&gt;0),(P6-G6)/G6,"")</f>
-        <v/>
-      </c>
-      <c r="S6" s="481">
-        <f>IF(AND(ISNUMBER(P6),P6&gt;0),IF(P6-G6&gt;0,"✅ กำไร","🔴 ขาดทุน"),"")</f>
-        <v/>
-      </c>
-      <c r="T6" s="482" t="n"/>
-      <c r="U6" s="482" t="n"/>
-      <c r="V6" s="482" t="n"/>
-      <c r="W6" s="482" t="n"/>
+      <c r="Q6" s="479" t="n"/>
+      <c r="R6" s="480" t="n"/>
+      <c r="S6" s="481" t="n"/>
     </row>
     <row r="7" ht="75" customHeight="1" s="350">
       <c r="A7" s="484" t="n"/>
@@ -8140,22 +8113,9 @@
       <c r="N7" s="497" t="n"/>
       <c r="O7" s="498" t="n"/>
       <c r="P7" s="478" t="n"/>
-      <c r="Q7" s="479">
-        <f>IF(AND(ISNUMBER(P7),P7&gt;0),P7-G7,"")</f>
-        <v/>
-      </c>
-      <c r="R7" s="480">
-        <f>IF(AND(ISNUMBER(P7),P7&gt;0),(P7-G7)/G7,"")</f>
-        <v/>
-      </c>
-      <c r="S7" s="481">
-        <f>IF(AND(ISNUMBER(P7),P7&gt;0),IF(P7-G7&gt;0,"✅ กำไร","🔴 ขาดทุน"),"")</f>
-        <v/>
-      </c>
-      <c r="T7" s="482" t="n"/>
-      <c r="U7" s="482" t="n"/>
-      <c r="V7" s="482" t="n"/>
-      <c r="W7" s="482" t="n"/>
+      <c r="Q7" s="479" t="n"/>
+      <c r="R7" s="480" t="n"/>
+      <c r="S7" s="481" t="n"/>
     </row>
     <row r="8" ht="75" customHeight="1" s="350">
       <c r="A8" s="484" t="n"/>
@@ -8186,10 +8146,6 @@
         <f>IF(AND(ISNUMBER(P8),P8&gt;0),IF(P8-G8&gt;0,"✅ กำไร","🔴 ขาดทุน"),"")</f>
         <v/>
       </c>
-      <c r="T8" s="482" t="n"/>
-      <c r="U8" s="482" t="n"/>
-      <c r="V8" s="482" t="n"/>
-      <c r="W8" s="482" t="n"/>
     </row>
     <row r="9" ht="75" customHeight="1" s="350">
       <c r="A9" s="484" t="n"/>
@@ -8220,10 +8176,6 @@
         <f>IF(AND(ISNUMBER(P9),P9&gt;0),IF(P9-G9&gt;0,"✅ กำไร","🔴 ขาดทุน"),"")</f>
         <v/>
       </c>
-      <c r="T9" s="482" t="n"/>
-      <c r="U9" s="482" t="n"/>
-      <c r="V9" s="482" t="n"/>
-      <c r="W9" s="482" t="n"/>
     </row>
     <row r="10" ht="24" customHeight="1" s="350">
       <c r="A10" s="499" t="inlineStr">
@@ -8281,12 +8233,7 @@
         <f>IF(SUM(Q4:Q9)&gt;0,"✅ กำไรรวม","🔴 ขาดทุนรวม")</f>
         <v/>
       </c>
-      <c r="T10" s="510" t="n"/>
-      <c r="U10" s="510" t="n"/>
-      <c r="V10" s="510" t="n"/>
-      <c r="W10" s="511" t="n"/>
-    </row>
-    <row r="11"/>
+    </row>
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="L2:M2"/>

</xml_diff>

<commit_message>
fix: PLTR price correction + homepage shows only portfolio stocks
- Fix PLTR price in Excel: $154 → $150.68 (22 มี.ค.)
- Fix read_portfolio() to cap at row 25 — excludes ผลรวม rows,
  comparison section, and หุ้นน่าจับตามอง watchlist (DELL, MU, QCOM)
- Rebuild index.html: homepage now shows exactly 20 stocks

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/รายรับ_รายจ่าย_ประจำปี.xlsx
+++ b/รายรับ_รายจ่าย_ประจำปี.xlsx
@@ -6261,7 +6261,7 @@
         <v>145.7341</v>
       </c>
       <c r="D11" s="367" t="n">
-        <v>154</v>
+        <v>150.68</v>
       </c>
       <c r="E11" s="368">
         <f>IF(D11&gt;0,G11*(D11-C11)/D11,0)</f>
@@ -6286,7 +6286,7 @@
       <c r="J11" s="373" t="n"/>
       <c r="K11" s="374" t="inlineStr">
         <is>
-          <t>🆕 21 มี.ค.</t>
+          <t>🆕 22 มี.ค.</t>
         </is>
       </c>
       <c r="L11" s="354" t="n"/>

</xml_diff>